<commit_message>
Add seven CB candidates to the pipeline workbook for video work
Joe Wright, Kaelan Casey, Jack Whatmough, Lee Jenkins, Matty Pearson,
Rarmani Edmonds-Green and Joe Low on the CB tab with club, 26/27 minutes
and fit notes; Progress left blank. Drop the Live Watchlist wording from
each tab's info line.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X8kAY4q3jCmdEW7FdbGNyy
</commit_message>
<xml_diff>
--- a/BRFC_Recruitment_Pipeline/BRFC_Recruitment_Pipeline.xlsx
+++ b/BRFC_Recruitment_Pipeline/BRFC_Recruitment_Pipeline.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CB" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GK" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CM 6" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LB" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Winger" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CM 8" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CM 10" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RB" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CF Target" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CF Runner" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="CB" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="GK" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="CM 6" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="LB" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Winger" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="CM 8" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="CM 10" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="RB" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="CF Target" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="CF Runner" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -105,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -127,6 +127,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -580,10 +583,11 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Players are added only after Dhillon agrees.  Progress = Y after video → Monday 'CB List' shortlist + Live Watchlist.</t>
-        </is>
-      </c>
-    </row>
+          <t>Players are added only after Dhillon agrees.  Progress = Y after video → Monday 'CB List' shortlist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -612,52 +616,150 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="7" t="n"/>
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Joe Wright</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Dundee</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="n">
+        <v>34</v>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>31, R foot. Fit 66.6 (24/25) → 78.2 (25/26), aerial + press. Low mins in SPL. Long List, no reports yet.</t>
+        </is>
+      </c>
       <c r="E11" s="6" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="n"/>
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="6" t="n"/>
-      <c r="D12" s="7" t="n"/>
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Kaelan Casey</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Stevenage (loan from West Ham)</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>331</v>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>20, RCB. Fit 73.0 (25/26), aerial. Loan target. Graded A - Sign, no report on file.</t>
+        </is>
+      </c>
       <c r="E12" s="6" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="n"/>
-      <c r="B13" s="5" t="n"/>
-      <c r="C13" s="6" t="n"/>
-      <c r="D13" s="7" t="n"/>
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Jack Whatmough</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Huddersfield Town</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>30. Fit 67.7 (24/25 only), aerial + press. Low mins in L1, out of contract 2027. B - Monitor Now.</t>
+        </is>
+      </c>
       <c r="E13" s="6" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="n"/>
-      <c r="B14" s="5" t="n"/>
-      <c r="C14" s="6" t="n"/>
-      <c r="D14" s="7" t="n"/>
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Lee Jenkins</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Newport County</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="n">
+        <v>880</v>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>24, L foot. Fit 56.6 (25/26) → 39.8 (26/27). Live watch Sep 25: aggressive, good in the air. No report. Already on Short List.</t>
+        </is>
+      </c>
       <c r="E14" s="6" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="n"/>
-      <c r="B15" s="5" t="n"/>
-      <c r="C15" s="6" t="n"/>
-      <c r="D15" s="7" t="n"/>
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Matty Pearson</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Doncaster Rovers</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>33, R foot. Fit 63.0 → 70.5. Video report Jan 26: aerial, set pieces, interceptions; composure under press weak. OOC 2027. Already on Short List.</t>
+        </is>
+      </c>
       <c r="E15" s="6" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="n"/>
-      <c r="B16" s="5" t="n"/>
-      <c r="C16" s="6" t="n"/>
-      <c r="D16" s="7" t="n"/>
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Rarmani Edmonds-Green</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Leyton Orient</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>27, RCB. Fit 58.5 (24/25, no sample since). 0 mins this season, out of contract 2027, marked Of Interest.</t>
+        </is>
+      </c>
       <c r="E16" s="6" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="n"/>
-      <c r="B17" s="5" t="n"/>
-      <c r="C17" s="6" t="n"/>
-      <c r="D17" s="7" t="n"/>
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Joe Low</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Huddersfield Town</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>24, mostly RCB. Fit 35.3 / 35.7 - low, no aerial or press tags. Low mins in L1.</t>
+        </is>
+      </c>
       <c r="E17" s="6" t="n"/>
     </row>
     <row r="18">
@@ -1036,8 +1138,8 @@
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A7:E7"/>
+    <mergeCell ref="A5:E5"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
     <mergeCell ref="A8:E8"/>
     <mergeCell ref="A6:E6"/>
     <mergeCell ref="A3:E3"/>
@@ -1114,10 +1216,11 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Players are added only after Dhillon agrees.  Progress = Y after video → Monday 'CF - Type B (Runner)' shortlist + Live Watchlist.</t>
-        </is>
-      </c>
-    </row>
+          <t>Players are added only after Dhillon agrees.  Progress = Y after video → Monday 'CF - Type B (Runner)' shortlist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
@@ -1653,10 +1756,11 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Players are added only after Dhillon agrees.  Progress = Y after video → Monday 'GK Lists' shortlist + Live Watchlist.</t>
-        </is>
-      </c>
-    </row>
+          <t>Players are added only after Dhillon agrees.  Progress = Y after video → Monday 'GK Lists' shortlist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
@@ -2109,8 +2213,8 @@
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A7:E7"/>
+    <mergeCell ref="A5:E5"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
     <mergeCell ref="A6:E6"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
@@ -2193,10 +2297,11 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Players are added only after Dhillon agrees.  Progress = Y after video → Monday 'CM - 6' shortlist + Live Watchlist.</t>
-        </is>
-      </c>
-    </row>
+          <t>Players are added only after Dhillon agrees.  Progress = Y after video → Monday 'CM - 6' shortlist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
@@ -2649,8 +2754,8 @@
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A7:E7"/>
+    <mergeCell ref="A5:E5"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
     <mergeCell ref="A6:E6"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
@@ -2733,10 +2838,11 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Players are added only after Dhillon agrees.  Progress = Y after video → Monday 'LB List' shortlist + Live Watchlist.</t>
-        </is>
-      </c>
-    </row>
+          <t>Players are added only after Dhillon agrees.  Progress = Y after video → Monday 'LB List' shortlist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
@@ -3189,8 +3295,8 @@
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A7:E7"/>
+    <mergeCell ref="A5:E5"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
     <mergeCell ref="A6:E6"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
@@ -3273,10 +3379,11 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Players are added only after Dhillon agrees.  Progress = Y after video → Monday 'Winger List' shortlist + Live Watchlist.</t>
-        </is>
-      </c>
-    </row>
+          <t>Players are added only after Dhillon agrees.  Progress = Y after video → Monday 'Winger List' shortlist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
@@ -3729,8 +3836,8 @@
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A7:E7"/>
+    <mergeCell ref="A5:E5"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
     <mergeCell ref="A6:E6"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
@@ -3813,10 +3920,11 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Players are added only after Dhillon agrees.  Progress = Y after video → Monday 'CM - 8' shortlist + Live Watchlist.</t>
-        </is>
-      </c>
-    </row>
+          <t>Players are added only after Dhillon agrees.  Progress = Y after video → Monday 'CM - 8' shortlist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
@@ -4269,8 +4377,8 @@
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A7:E7"/>
+    <mergeCell ref="A5:E5"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
     <mergeCell ref="A6:E6"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
@@ -4353,10 +4461,11 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Players are added only after Dhillon agrees.  Progress = Y after video → Monday 'CM - 10' shortlist + Live Watchlist.</t>
-        </is>
-      </c>
-    </row>
+          <t>Players are added only after Dhillon agrees.  Progress = Y after video → Monday 'CM - 10' shortlist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
@@ -4809,8 +4918,8 @@
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A7:E7"/>
+    <mergeCell ref="A5:E5"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
     <mergeCell ref="A6:E6"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
@@ -4893,10 +5002,11 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Players are added only after Dhillon agrees.  Progress = Y after video → Monday 'RB List' shortlist + Live Watchlist.</t>
-        </is>
-      </c>
-    </row>
+          <t>Players are added only after Dhillon agrees.  Progress = Y after video → Monday 'RB List' shortlist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
@@ -5349,8 +5459,8 @@
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A7:E7"/>
+    <mergeCell ref="A5:E5"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
     <mergeCell ref="A6:E6"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
@@ -5426,10 +5536,11 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Players are added only after Dhillon agrees.  Progress = Y after video → Monday 'CF - Type A (Target)' shortlist + Live Watchlist.</t>
-        </is>
-      </c>
-    </row>
+          <t>Players are added only after Dhillon agrees.  Progress = Y after video → Monday 'CF - Type A (Target)' shortlist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Leave CB Notes column empty for scouts
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X8kAY4q3jCmdEW7FdbGNyy
</commit_message>
<xml_diff>
--- a/BRFC_Recruitment_Pipeline/BRFC_Recruitment_Pipeline.xlsx
+++ b/BRFC_Recruitment_Pipeline/BRFC_Recruitment_Pipeline.xlsx
@@ -587,7 +587,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -629,11 +628,7 @@
       <c r="C11" s="8" t="n">
         <v>34</v>
       </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>31, R foot. Fit 66.6 (24/25) → 78.2 (25/26), aerial + press. Low mins in SPL. Long List, no reports yet.</t>
-        </is>
-      </c>
+      <c r="D11" s="8" t="n"/>
       <c r="E11" s="6" t="n"/>
     </row>
     <row r="12">
@@ -650,11 +645,7 @@
       <c r="C12" s="8" t="n">
         <v>331</v>
       </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>20, RCB. Fit 73.0 (25/26), aerial. Loan target. Graded A - Sign, no report on file.</t>
-        </is>
-      </c>
+      <c r="D12" s="8" t="n"/>
       <c r="E12" s="6" t="n"/>
     </row>
     <row r="13">
@@ -671,11 +662,7 @@
       <c r="C13" s="8" t="n">
         <v>97</v>
       </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>30. Fit 67.7 (24/25 only), aerial + press. Low mins in L1, out of contract 2027. B - Monitor Now.</t>
-        </is>
-      </c>
+      <c r="D13" s="8" t="n"/>
       <c r="E13" s="6" t="n"/>
     </row>
     <row r="14">
@@ -692,11 +679,7 @@
       <c r="C14" s="8" t="n">
         <v>880</v>
       </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>24, L foot. Fit 56.6 (25/26) → 39.8 (26/27). Live watch Sep 25: aggressive, good in the air. No report. Already on Short List.</t>
-        </is>
-      </c>
+      <c r="D14" s="8" t="n"/>
       <c r="E14" s="6" t="n"/>
     </row>
     <row r="15">
@@ -713,11 +696,7 @@
       <c r="C15" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>33, R foot. Fit 63.0 → 70.5. Video report Jan 26: aerial, set pieces, interceptions; composure under press weak. OOC 2027. Already on Short List.</t>
-        </is>
-      </c>
+      <c r="D15" s="8" t="n"/>
       <c r="E15" s="6" t="n"/>
     </row>
     <row r="16">
@@ -734,11 +713,7 @@
       <c r="C16" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>27, RCB. Fit 58.5 (24/25, no sample since). 0 mins this season, out of contract 2027, marked Of Interest.</t>
-        </is>
-      </c>
+      <c r="D16" s="8" t="n"/>
       <c r="E16" s="6" t="n"/>
     </row>
     <row r="17">
@@ -755,11 +730,7 @@
       <c r="C17" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>24, mostly RCB. Fit 35.3 / 35.7 - low, no aerial or press tags. Low mins in L1.</t>
-        </is>
-      </c>
+      <c r="D17" s="8" t="n"/>
       <c r="E17" s="6" t="n"/>
     </row>
     <row r="18">
@@ -1220,7 +1191,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
@@ -1760,7 +1730,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
@@ -2301,7 +2270,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
@@ -2842,7 +2810,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
@@ -3383,7 +3350,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
@@ -3924,7 +3890,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
@@ -4465,7 +4430,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
@@ -5006,7 +4970,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
@@ -5540,7 +5503,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>

</xml_diff>